<commit_message>
Ordered by is now a column on each order line; Airco navy/orange colors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/2250823/2250823_AUSTINSTONE_OpenQuestions.xlsx
+++ b/tracker/2250823/2250823_AUSTINSTONE_OpenQuestions.xlsx
@@ -29,7 +29,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="002B3C8E"/>
       <sz val="16"/>
     </font>
     <font>
@@ -49,12 +49,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00DCE0F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="002B3C8E"/>
       </patternFill>
     </fill>
     <fill>
@@ -68,13 +68,18 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00FC7C36"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -90,32 +95,47 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FC7C36"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -497,353 +517,355 @@
           <t>OPEN QUESTIONS</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Job number</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>2250823</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Project name</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Austin Stone</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Airco PM</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>4 open - ready to send when this is 0 and every unit and filter is accounted for</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Who knows</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>All 7 RTUs need 84 filters, only 72 ordered: one RTU's worth (12) short overall. Either 1 of the 2" RTUs (1A, 2A, 1C, 2C) still needs 2" (8 of 20x25x2 + 4 of 20x20x2), or a 2" unit got 4" and RTU-2B-1 will be short on 4". Which units got what size?</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Angel / techs</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>For each order, which units did the filters go to (fills the 'Units it went to' column)?</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Techs</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>When will RTU-2B-1 be started? The extra 12 4" filters ordered are on hand for it unless they were used as substitutes.</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>AHU-1 and ERV-1 are not replaced yet. Are their sizes right (20x24 vs the RTUs' 20x25)? Set 3 must match the spec size exactly.</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Angel / PM</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>RTU-2B-1 (not 2B-2) is the one RTU not started up yet. 6 of 7 RTUs replaced.</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Phase: none right now. Added scope may come as a phase on this job number or a new job number; jobs are always separated by job number.</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Attic stock: none planned. The PM can add it at any time (MERV 13).</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>AHU-1 and ERV-1 not replaced yet.</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>PO numbers: 380118 for the 12-filter order, 382244 for the 60-filter order.</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Order 1 date is 9/22/2026 (not 9/25).</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Both orders are Set 2, MERV 8.</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Angel</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="9" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="9" t="n"/>
+      <c r="C25" s="9" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="n"/>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="9" t="n"/>
+      <c r="C27" s="9" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="n"/>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="n"/>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="9" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="n"/>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="n"/>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="9" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="n"/>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="n"/>
-      <c r="B35" s="8" t="n"/>
-      <c r="C35" s="8" t="n"/>
+      <c r="A35" s="11" t="n"/>
+      <c r="B35" s="9" t="n"/>
+      <c r="C35" s="9" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="n"/>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
+      <c r="A37" s="11" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>